<commit_message>
generation of souffle executables and measuring 10 runs of each executable
</commit_message>
<xml_diff>
--- a/benchmark/functional/powdataflow/dataflow-measurements.xlsx
+++ b/benchmark/functional/powdataflow/dataflow-measurements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andiderp/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89621A02-AE2F-A44D-8214-8BBCE50C75A7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E457C55E-078A-404D-9F61-CA319C5F6C81}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" activeTab="5" xr2:uid="{C47F41CB-B47E-0148-87C7-130387C9F0E8}"/>
+    <workbookView xWindow="19480" yWindow="660" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{C47F41CB-B47E-0148-87C7-130387C9F0E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Formulog" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="24">
   <si>
     <t>Ex1 (ms)</t>
   </si>
@@ -74,6 +74,42 @@
   </si>
   <si>
     <t>Ex4 Insert (ms)</t>
+  </si>
+  <si>
+    <t>Ex1 real (ms)</t>
+  </si>
+  <si>
+    <t>Ex1 user (ms)</t>
+  </si>
+  <si>
+    <t>Ex1 sys (ms)</t>
+  </si>
+  <si>
+    <t>Ex2 real (ms)</t>
+  </si>
+  <si>
+    <t>Ex2 user (ms)</t>
+  </si>
+  <si>
+    <t>Ex2 sys (ms)</t>
+  </si>
+  <si>
+    <t>Ex3 real (ms)</t>
+  </si>
+  <si>
+    <t>Ex3 user (ms)</t>
+  </si>
+  <si>
+    <t>Ex3 sys (ms)</t>
+  </si>
+  <si>
+    <t>Ex4 real (ms)</t>
+  </si>
+  <si>
+    <t>Ex4 user (ms)</t>
+  </si>
+  <si>
+    <t>Ex4 sys (ms)</t>
   </si>
 </sst>
 </file>
@@ -1858,21 +1894,425 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8E3DE85-AD94-AB43-91C3-A301AEC98FD3}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>247</v>
+      </c>
+      <c r="B2">
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>248</v>
+      </c>
+      <c r="E2">
+        <v>87</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>240</v>
+      </c>
+      <c r="H2">
+        <v>23</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>265</v>
+      </c>
+      <c r="K2">
+        <v>73</v>
+      </c>
+      <c r="L2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>16</v>
+      </c>
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D3">
+        <v>93</v>
+      </c>
+      <c r="E3">
+        <v>88</v>
+      </c>
+      <c r="F3">
         <v>3</v>
+      </c>
+      <c r="G3">
+        <v>24</v>
+      </c>
+      <c r="H3">
+        <v>21</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>77</v>
+      </c>
+      <c r="K3">
+        <v>73</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>19</v>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>93</v>
+      </c>
+      <c r="E4">
+        <v>89</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>24</v>
+      </c>
+      <c r="H4">
+        <v>21</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>79</v>
+      </c>
+      <c r="K4">
+        <v>74</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>19</v>
+      </c>
+      <c r="B5">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>94</v>
+      </c>
+      <c r="E5">
+        <v>89</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>24</v>
+      </c>
+      <c r="H5">
+        <v>21</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>81</v>
+      </c>
+      <c r="K5">
+        <v>75</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>96</v>
+      </c>
+      <c r="E6">
+        <v>91</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6">
+        <v>21</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>117</v>
+      </c>
+      <c r="K6">
+        <v>96</v>
+      </c>
+      <c r="L6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>16</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>97</v>
+      </c>
+      <c r="E7">
+        <v>91</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <v>21</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>109</v>
+      </c>
+      <c r="K7">
+        <v>89</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>19</v>
+      </c>
+      <c r="B8">
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>94</v>
+      </c>
+      <c r="E8">
+        <v>89</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>24</v>
+      </c>
+      <c r="H8">
+        <v>21</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8">
+        <v>85</v>
+      </c>
+      <c r="K8">
+        <v>78</v>
+      </c>
+      <c r="L8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>19</v>
+      </c>
+      <c r="B9">
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>94</v>
+      </c>
+      <c r="E9">
+        <v>89</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>24</v>
+      </c>
+      <c r="H9">
+        <v>21</v>
+      </c>
+      <c r="I9">
+        <v>2</v>
+      </c>
+      <c r="J9">
+        <v>85</v>
+      </c>
+      <c r="K9">
+        <v>78</v>
+      </c>
+      <c r="L9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>19</v>
+      </c>
+      <c r="B10">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>97</v>
+      </c>
+      <c r="E10">
+        <v>91</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
+        <v>24</v>
+      </c>
+      <c r="H10">
+        <v>21</v>
+      </c>
+      <c r="I10">
+        <v>2</v>
+      </c>
+      <c r="J10">
+        <v>93</v>
+      </c>
+      <c r="K10">
+        <v>82</v>
+      </c>
+      <c r="L10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>19</v>
+      </c>
+      <c r="B11">
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>97</v>
+      </c>
+      <c r="E11">
+        <v>90</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <v>24</v>
+      </c>
+      <c r="H11">
+        <v>21</v>
+      </c>
+      <c r="I11">
+        <v>2</v>
+      </c>
+      <c r="J11">
+        <v>87</v>
+      </c>
+      <c r="K11">
+        <v>79</v>
+      </c>
+      <c r="L11">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1882,20 +2322,427 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65CCEC3C-B1DC-7141-A7D8-9D622D2B31EC}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>23</v>
+      </c>
+      <c r="B2">
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>147</v>
+      </c>
+      <c r="E2">
+        <v>128</v>
+      </c>
+      <c r="F2">
+        <v>7</v>
+      </c>
+      <c r="G2">
+        <v>252</v>
+      </c>
+      <c r="H2">
+        <v>45</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>246</v>
+      </c>
+      <c r="K2">
+        <v>52</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>21</v>
+      </c>
+      <c r="B3">
+        <v>18</v>
+      </c>
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D3">
+        <v>120</v>
+      </c>
+      <c r="E3">
+        <v>114</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>49</v>
+      </c>
+      <c r="H3">
+        <v>44</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>56</v>
+      </c>
+      <c r="K3">
+        <v>52</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>21</v>
+      </c>
+      <c r="B4">
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>120</v>
+      </c>
+      <c r="E4">
+        <v>115</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>50</v>
+      </c>
+      <c r="H4">
+        <v>45</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>56</v>
+      </c>
+      <c r="K4">
+        <v>52</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>21</v>
+      </c>
+      <c r="B5">
+        <v>18</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>122</v>
+      </c>
+      <c r="E5">
+        <v>116</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>50</v>
+      </c>
+      <c r="H5">
+        <v>45</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>58</v>
+      </c>
+      <c r="K5">
+        <v>52</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>21</v>
+      </c>
+      <c r="B6">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>116</v>
+      </c>
+      <c r="E6">
+        <v>112</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6">
+        <v>50</v>
+      </c>
+      <c r="H6">
+        <v>45</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>56</v>
+      </c>
+      <c r="K6">
+        <v>51</v>
+      </c>
+      <c r="L6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>21</v>
+      </c>
+      <c r="B7">
+        <v>18</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>117</v>
+      </c>
+      <c r="E7">
+        <v>113</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>49</v>
+      </c>
+      <c r="H7">
+        <v>44</v>
+      </c>
+      <c r="I7">
+        <v>3</v>
+      </c>
+      <c r="J7">
+        <v>59</v>
+      </c>
+      <c r="K7">
+        <v>53</v>
+      </c>
+      <c r="L7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>18</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>119</v>
+      </c>
+      <c r="E8">
+        <v>114</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="G8">
+        <v>48</v>
+      </c>
+      <c r="H8">
+        <v>44</v>
+      </c>
+      <c r="I8">
+        <v>3</v>
+      </c>
+      <c r="J8">
+        <v>59</v>
+      </c>
+      <c r="K8">
+        <v>53</v>
+      </c>
+      <c r="L8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>18</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>120</v>
+      </c>
+      <c r="E9">
+        <v>115</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="G9">
+        <v>49</v>
+      </c>
+      <c r="H9">
+        <v>45</v>
+      </c>
+      <c r="I9">
+        <v>3</v>
+      </c>
+      <c r="J9">
+        <v>62</v>
+      </c>
+      <c r="K9">
+        <v>55</v>
+      </c>
+      <c r="L9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>19</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>118</v>
+      </c>
+      <c r="E10">
+        <v>113</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>49</v>
+      </c>
+      <c r="H10">
+        <v>44</v>
+      </c>
+      <c r="I10">
+        <v>3</v>
+      </c>
+      <c r="J10">
+        <v>60</v>
+      </c>
+      <c r="K10">
+        <v>53</v>
+      </c>
+      <c r="L10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>21</v>
+      </c>
+      <c r="B11">
+        <v>17</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>117</v>
+      </c>
+      <c r="E11">
+        <v>112</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>52</v>
+      </c>
+      <c r="H11">
+        <v>46</v>
+      </c>
+      <c r="I11">
+        <v>3</v>
+      </c>
+      <c r="J11">
+        <v>59</v>
+      </c>
+      <c r="K11">
+        <v>53</v>
+      </c>
+      <c r="L11">
         <v>3</v>
       </c>
     </row>

</xml_diff>